<commit_message>
cleaning up and adding comments to wave model scripts
</commit_message>
<xml_diff>
--- a/validation/umwm_wind_waveheights.xlsx
+++ b/validation/umwm_wind_waveheights.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5d40ba198affbc6f/Desktop/Main/Work/Github_Repos/umwm_titan/validation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\OneDrive\Documents\00_Main\Work\Github_Repos\PlanetWaves\validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="216" documentId="8_{1ECAA66D-5BF5-4A0F-8594-AA91DC5B4E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{590B6DCA-57CD-4939-9D88-967DF9D764BD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF525E8-31BB-4917-85CC-88D33DDCA252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="18192" windowHeight="11472" xr2:uid="{606F5AC5-7EA0-4448-AE08-6084F6885092}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>u</t>
   </si>
@@ -50,20 +50,36 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>with zeroingline 437</t>
+    <t>old</t>
+  </si>
+  <si>
+    <t>new</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -86,8 +102,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -103,10 +126,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -426,10 +445,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8806629-2C9F-469E-B362-0412F78F93CE}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -439,308 +458,474 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B3" s="1">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>0</v>
       </c>
       <c r="C4">
-        <v>3.0421299999999998E-2</v>
-      </c>
-      <c r="D4">
-        <v>3.0425600000000001E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>8.1498347222804995E-2</v>
       </c>
       <c r="C5">
-        <v>0.14451800000000001</v>
-      </c>
-      <c r="D5">
-        <v>0.14466300000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>5.8842584490776E-2</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="N5" t="s">
+        <v>4</v>
+      </c>
+      <c r="O5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>0.18736366927623699</v>
       </c>
       <c r="C6">
-        <v>0.26693800000000001</v>
-      </c>
-      <c r="D6">
-        <v>0.26702199999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>0.16594126820564201</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="N6" s="2">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>0.319779723882675</v>
       </c>
       <c r="C7">
-        <v>0.43732599999999999</v>
-      </c>
-      <c r="D7">
-        <v>0.43737599999999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>0.29799547791481001</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="N7" s="2">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>6</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>0.48304304480552601</v>
       </c>
       <c r="C8">
-        <v>0.64294499999999999</v>
-      </c>
-      <c r="D8">
-        <v>0.64298900000000003</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>0.45951050519943198</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="N8" s="2">
+        <v>3.0421E-2</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>7</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>0.67869186401367099</v>
       </c>
       <c r="C9">
-        <v>0.87729599999999996</v>
-      </c>
-      <c r="D9">
-        <v>0.87731800000000004</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>0.65201592445373502</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="N9" s="2">
+        <v>0.14451800000000001</v>
+      </c>
+      <c r="O9">
+        <v>5.8842584490776E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>8</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>0.90832310914993197</v>
       </c>
       <c r="C10">
-        <v>1.14096</v>
-      </c>
-      <c r="D10">
-        <v>1.1409499999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>0.87661045789718595</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="N10" s="2">
+        <v>0.26693800000000001</v>
+      </c>
+      <c r="O10">
+        <v>0.16594126820564201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>9</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>1.1727869510650599</v>
       </c>
       <c r="C11">
-        <v>1.4317200000000001</v>
-      </c>
-      <c r="D11">
-        <v>1.43167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>1.13389360904693</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="N11" s="2">
+        <v>0.43732599999999999</v>
+      </c>
+      <c r="O11">
+        <v>0.29799547791481001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>10</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>1.47175681591033</v>
       </c>
       <c r="C12">
-        <v>1.7474400000000001</v>
-      </c>
-      <c r="D12">
-        <v>1.7473399999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>1.42357325553894</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="N12" s="2">
+        <v>0.64294499999999999</v>
+      </c>
+      <c r="O12">
+        <v>0.45951050519943198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>11</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>1.80442786216735</v>
       </c>
       <c r="C13">
-        <v>2.0729600000000001</v>
-      </c>
-      <c r="D13">
-        <v>2.0727799999999998</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>1.74535477161407</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="N13" s="2">
+        <v>0.87729599999999996</v>
+      </c>
+      <c r="O13">
+        <v>0.65201592445373502</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>12</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>2.1610410213470401</v>
       </c>
       <c r="C14">
-        <v>2.42971</v>
-      </c>
-      <c r="D14">
-        <v>2.4294500000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>2.0883898735046298</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="N14" s="2">
+        <v>1.14096</v>
+      </c>
+      <c r="O14">
+        <v>0.87661045789718595</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>13</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>2.5583541393279998</v>
       </c>
       <c r="C15">
-        <v>2.7871100000000002</v>
-      </c>
-      <c r="D15">
-        <v>2.7867500000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>2.4712917804718</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="N15" s="2">
+        <v>1.4317200000000001</v>
+      </c>
+      <c r="O15">
+        <v>1.13389360904693</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>14</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>2.98986363410949</v>
       </c>
       <c r="C16">
-        <v>3.1803699999999999</v>
-      </c>
-      <c r="D16">
-        <v>3.17991</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>2.8871443271636901</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="N16" s="2">
+        <v>1.7474400000000001</v>
+      </c>
+      <c r="O16">
+        <v>1.42357325553894</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>15</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>3.4347374439239502</v>
       </c>
       <c r="C17">
-        <v>3.5927699999999998</v>
-      </c>
-      <c r="D17">
-        <v>3.5922200000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>3.3141736984252899</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="N17" s="2">
+        <v>2.0729600000000001</v>
+      </c>
+      <c r="O17">
+        <v>1.74535477161407</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>16</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <v>3.93021535873413</v>
       </c>
       <c r="C18">
-        <v>3.9786000000000001</v>
-      </c>
-      <c r="D18">
-        <v>3.9779399999999998</v>
-      </c>
+        <v>3.7912406921386701</v>
+      </c>
+      <c r="D18" s="1"/>
       <c r="E18" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="N18" s="2">
+        <v>2.42971</v>
+      </c>
+      <c r="O18">
+        <v>2.0883898735046298</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>17</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="1">
         <v>4.4217596054077104</v>
       </c>
       <c r="C19">
-        <v>4.3825599999999998</v>
-      </c>
-      <c r="D19">
-        <v>4.3818000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>4.2632799148559499</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="N19" s="2">
+        <v>2.7871100000000002</v>
+      </c>
+      <c r="O19">
+        <v>2.4712917804718</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>18</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="1">
         <v>4.9297094345092702</v>
       </c>
       <c r="C20">
-        <v>4.8433299999999999</v>
-      </c>
-      <c r="D20">
-        <v>4.8424800000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>4.7498655319213796</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="N20" s="2">
+        <v>3.1803699999999999</v>
+      </c>
+      <c r="O20">
+        <v>2.8871443271636901</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>19</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="1">
         <v>5.4979319572448704</v>
       </c>
       <c r="C21">
-        <v>5.2761300000000002</v>
-      </c>
-      <c r="D21">
-        <v>5.2751700000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>5.2975568771362296</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="N21" s="2">
+        <v>3.5927699999999998</v>
+      </c>
+      <c r="O21">
+        <v>3.3141736984252899</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>20</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="1">
         <v>6.0374197959899902</v>
       </c>
       <c r="C22">
+        <v>5.8154425621032697</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="N22" s="2">
+        <v>3.9786000000000001</v>
+      </c>
+      <c r="O22">
+        <v>3.7912406921386701</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="N23" s="2">
+        <v>4.3825599999999998</v>
+      </c>
+      <c r="O23">
+        <v>4.2632799148559499</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="N24" s="2">
+        <v>4.8433299999999999</v>
+      </c>
+      <c r="O24">
+        <v>4.7498655319213796</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="N25" s="2">
+        <v>5.2761300000000002</v>
+      </c>
+      <c r="O25">
+        <v>5.2975568771362296</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="N26" s="2">
         <v>5.77555</v>
       </c>
-      <c r="D22">
-        <v>5.7745300000000004</v>
+      <c r="O26">
+        <v>5.8154425621032697</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cleaning up validation folder for generic user
-changed absolute file path to relative file path
-reorganized the validation folder so all relevant scripts are within one folder
-
</commit_message>
<xml_diff>
--- a/validation/umwm_wind_waveheights.xlsx
+++ b/validation/umwm_wind_waveheights.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\OneDrive\Documents\00_Main\Work\Github_Repos\PlanetWaves\validation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5d40ba198affbc6f/Documents/00_Main/Work/Github_Repos/PlanetWaves/validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF525E8-31BB-4917-85CC-88D33DDCA252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2AF525E8-31BB-4917-85CC-88D33DDCA252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4646CFC-0427-4B74-B05A-A778A9685441}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="18192" windowHeight="11472" xr2:uid="{606F5AC5-7EA0-4448-AE08-6084F6885092}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="18000" windowHeight="10920" xr2:uid="{606F5AC5-7EA0-4448-AE08-6084F6885092}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>u</t>
   </si>
@@ -48,12 +48,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>old</t>
-  </si>
-  <si>
-    <t>new</t>
   </si>
 </sst>
 </file>
@@ -445,10 +439,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8806629-2C9F-469E-B362-0412F78F93CE}">
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -460,7 +454,7 @@
       </c>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>0</v>
       </c>
@@ -473,7 +467,7 @@
       <c r="D2" s="1"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>1</v>
       </c>
@@ -486,7 +480,7 @@
       <c r="D3" s="1"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>2</v>
       </c>
@@ -499,7 +493,7 @@
       <c r="D4" s="1"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>3</v>
       </c>
@@ -513,14 +507,8 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="N5" t="s">
-        <v>4</v>
-      </c>
-      <c r="O5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>4</v>
       </c>
@@ -534,14 +522,8 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
-      <c r="N6" s="2">
-        <v>0</v>
-      </c>
-      <c r="O6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>5</v>
       </c>
@@ -555,14 +537,8 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
-      <c r="N7" s="2">
-        <v>0</v>
-      </c>
-      <c r="O7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>6</v>
       </c>
@@ -576,14 +552,8 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
-      <c r="N8" s="2">
-        <v>3.0421E-2</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>7</v>
       </c>
@@ -597,14 +567,8 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
-      <c r="N9" s="2">
-        <v>0.14451800000000001</v>
-      </c>
-      <c r="O9">
-        <v>5.8842584490776E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>8</v>
       </c>
@@ -618,14 +582,8 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
-      <c r="N10" s="2">
-        <v>0.26693800000000001</v>
-      </c>
-      <c r="O10">
-        <v>0.16594126820564201</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>9</v>
       </c>
@@ -639,14 +597,8 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
-      <c r="N11" s="2">
-        <v>0.43732599999999999</v>
-      </c>
-      <c r="O11">
-        <v>0.29799547791481001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>10</v>
       </c>
@@ -660,14 +612,8 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
-      <c r="N12" s="2">
-        <v>0.64294499999999999</v>
-      </c>
-      <c r="O12">
-        <v>0.45951050519943198</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>11</v>
       </c>
@@ -681,14 +627,8 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
-      <c r="N13" s="2">
-        <v>0.87729599999999996</v>
-      </c>
-      <c r="O13">
-        <v>0.65201592445373502</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>12</v>
       </c>
@@ -702,14 +642,8 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
-      <c r="N14" s="2">
-        <v>1.14096</v>
-      </c>
-      <c r="O14">
-        <v>0.87661045789718595</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>13</v>
       </c>
@@ -723,14 +657,8 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
-      <c r="N15" s="2">
-        <v>1.4317200000000001</v>
-      </c>
-      <c r="O15">
-        <v>1.13389360904693</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>14</v>
       </c>
@@ -744,14 +672,8 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
-      <c r="N16" s="2">
-        <v>1.7474400000000001</v>
-      </c>
-      <c r="O16">
-        <v>1.42357325553894</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>15</v>
       </c>
@@ -765,14 +687,8 @@
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
-      <c r="N17" s="2">
-        <v>2.0729600000000001</v>
-      </c>
-      <c r="O17">
-        <v>1.74535477161407</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>16</v>
       </c>
@@ -789,14 +705,8 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
-      <c r="N18" s="2">
-        <v>2.42971</v>
-      </c>
-      <c r="O18">
-        <v>2.0883898735046298</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>17</v>
       </c>
@@ -810,14 +720,8 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
-      <c r="N19" s="2">
-        <v>2.7871100000000002</v>
-      </c>
-      <c r="O19">
-        <v>2.4712917804718</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>18</v>
       </c>
@@ -831,14 +735,8 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
-      <c r="N20" s="2">
-        <v>3.1803699999999999</v>
-      </c>
-      <c r="O20">
-        <v>2.8871443271636901</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>19</v>
       </c>
@@ -852,14 +750,8 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
-      <c r="N21" s="2">
-        <v>3.5927699999999998</v>
-      </c>
-      <c r="O21">
-        <v>3.3141736984252899</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>20</v>
       </c>
@@ -873,56 +765,26 @@
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
-      <c r="N22" s="2">
-        <v>3.9786000000000001</v>
-      </c>
-      <c r="O22">
-        <v>3.7912406921386701</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
-      <c r="N23" s="2">
-        <v>4.3825599999999998</v>
-      </c>
-      <c r="O23">
-        <v>4.2632799148559499</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="N24" s="2">
-        <v>4.8433299999999999</v>
-      </c>
-      <c r="O24">
-        <v>4.7498655319213796</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
-      <c r="N25" s="2">
-        <v>5.2761300000000002</v>
-      </c>
-      <c r="O25">
-        <v>5.2975568771362296</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
-      <c r="N26" s="2">
-        <v>5.77555</v>
-      </c>
-      <c r="O26">
-        <v>5.8154425621032697</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>